<commit_message>
reverted back to prev model
</commit_message>
<xml_diff>
--- a/09_Human_gaze_detection/Human_gaze_detection_cam/exe/resnet18_cam/resnet18_cam_summary.xlsx
+++ b/09_Human_gaze_detection/Human_gaze_detection_cam/exe/resnet18_cam/resnet18_cam_summary.xlsx
@@ -949,7 +949,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>192</t>
+          <t>/conv1/Conv_output_0</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>/maxpool/MaxPool_output_0</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1069,7 +1069,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>195</t>
+          <t>/layer1/layer1.0/conv1/Conv_output_0</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1129,7 +1129,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>198</t>
+          <t>/layer1/layer1.0/conv2/Conv_output_0</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>/layer1/layer1.0/Add_output_0</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1249,7 +1249,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>/layer1/layer1.1/conv1/Conv_output_0</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1309,7 +1309,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>204</t>
+          <t>/layer1/layer1.1/conv2/Conv_output_0</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1369,7 +1369,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>139</t>
+          <t>/layer1/layer1.1/Add_output_0</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1429,7 +1429,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>207</t>
+          <t>/layer2/layer2.0/conv1/Conv_output_0</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>/layer2/layer2.0/conv2/Conv_output_0</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1549,7 +1549,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>213</t>
+          <t>/layer2/layer2.0/downsample/downsample.0/Conv_output_0</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1609,7 +1609,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>/layer2/layer2.0/Add_output_0</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>216</t>
+          <t>/layer2/layer2.1/conv1/Conv_output_0</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>219</t>
+          <t>/layer2/layer2.1/conv2/Conv_output_0</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>155</t>
+          <t>/layer2/layer2.1/Add_output_0</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>222</t>
+          <t>/layer3/layer3.0/conv1/Conv_output_0</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1909,7 +1909,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>225</t>
+          <t>/layer3/layer3.0/conv2/Conv_output_0</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>228</t>
+          <t>/layer3/layer3.0/downsample/downsample.0/Conv_output_0</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -2029,7 +2029,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>164</t>
+          <t>/layer3/layer3.0/Add_output_0</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>231</t>
+          <t>/layer3/layer3.1/conv1/Conv_output_0</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>234</t>
+          <t>/layer3/layer3.1/conv2/Conv_output_0</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2209,7 +2209,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>171</t>
+          <t>/layer3/layer3.1/Add_output_0</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -2269,7 +2269,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>237</t>
+          <t>/layer4/layer4.0/conv1/Conv_output_0</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>240</t>
+          <t>/layer4/layer4.0/conv2/Conv_output_0</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>243</t>
+          <t>/layer4/layer4.0/downsample/downsample.0/Conv_output_0</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -2449,7 +2449,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>/layer4/layer4.0/Add_output_0</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>246</t>
+          <t>/layer4/layer4.1/conv1/Conv_output_0</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2569,7 +2569,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>249</t>
+          <t>/layer4/layer4.1/conv2/Conv_output_0</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2629,7 +2629,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>187</t>
+          <t>/layer4/layer4.1/Add_output_0</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2689,7 +2689,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>189</t>
+          <t>/global_pool/pool/GlobalAveragePool_output_0</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">

</xml_diff>